<commit_message>
simplification form chantier + counts vehicules
</commit_message>
<xml_diff>
--- a/field/hanoi_construction_form.xlsx
+++ b/field/hanoi_construction_form.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,16 +461,6 @@
           <t>hint</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>constraint</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>constraint_message</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -487,8 +477,6 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -505,8 +493,6 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -535,8 +521,6 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -551,7 +535,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Construction site location (stand at the edge of the site)</t>
+          <t>Construction site location (stand at the edge)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -562,11 +546,9 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Wait for accuracy &lt; 10 m</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+          <t>Then take 2-3 NORMAL measurements walking away — the radius is computed from those</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -595,8 +577,6 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -625,57 +605,43 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>db_at_edge</t>
+          <t>site_photo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>dB at the edge of the site (~5 m)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>Photo of the site</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>0</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>. &gt;= 20 and . &lt;= 120</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>20-120 dB</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>db_at_25m</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>dB at ~25 m</t>
+          <t>Description (what is being built/demolished, machinery...)</t>
         </is>
       </c>
       <c r="D9" t="b">
@@ -683,128 +649,6 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>. &gt;= 20 and . &lt;= 120</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>20-120 dB</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>db_at_50m</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>dB at ~50 m</t>
-        </is>
-      </c>
-      <c r="D10" t="b">
-        <v>0</v>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>. &gt;= 20 and . &lt;= 120</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>20-120 dB</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>db_at_100m</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>dB at ~100 m (skip if not audible anymore)</t>
-        </is>
-      </c>
-      <c r="D11" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>. &gt;= 20 and . &lt;= 120</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>20-120 dB</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>image</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>site_photo</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Photo of the site</t>
-        </is>
-      </c>
-      <c r="D12" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Description (what is being built/demolished, machinery...)</t>
-        </is>
-      </c>
-      <c r="D13" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1029,7 +873,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026061202</t>
+          <t>2026061203</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>